<commit_message>
trying to get co2 tax connected with pps
</commit_message>
<xml_diff>
--- a/SuppXLS/Scen_CO2_price.xlsx
+++ b/SuppXLS/Scen_CO2_price.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FA3D86E-E8D9-4477-A8AE-DCC0D5EA2C71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86F3D1C2-2CC4-4EAB-98CA-795028B2C2B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CO2" sheetId="1" r:id="rId1"/>
+    <sheet name="cite" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,10 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
-  <si>
-    <t>~TFM_INS-TS</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="23">
   <si>
     <t>TimeSlice</t>
   </si>
@@ -56,20 +54,68 @@
     <t>*</t>
   </si>
   <si>
-    <t>USD25/kt</t>
-  </si>
-  <si>
     <t>com_taxnet</t>
   </si>
   <si>
     <t>TOTCO2</t>
+  </si>
+  <si>
+    <t>Trends and projections in the EU-ETS in 2025.</t>
+  </si>
+  <si>
+    <t>EUR2023</t>
+  </si>
+  <si>
+    <t>EUR2025</t>
+  </si>
+  <si>
+    <t>USD24/tCO2</t>
+  </si>
+  <si>
+    <t>2024 avg usd to eur rate (eur/usd)</t>
+  </si>
+  <si>
+    <t>EUR24/tCO2</t>
+  </si>
+  <si>
+    <t>avg eur25 inflation rate (EU)</t>
+  </si>
+  <si>
+    <t>EUR25/Tco2</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>WEM-ETS</t>
+  </si>
+  <si>
+    <t>WAM-ETS</t>
+  </si>
+  <si>
+    <t>WOM-ETS</t>
+  </si>
+  <si>
+    <t>HICP_2023</t>
+  </si>
+  <si>
+    <t>HICP_2025</t>
+  </si>
+  <si>
+    <t>eur25/kt</t>
+  </si>
+  <si>
+    <t>~TFM_INS</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+  </numFmts>
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -95,6 +141,21 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -143,21 +204,32 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="3"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="4">
+    <cellStyle name="Hyperlink" xfId="3" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 3" xfId="1" xr:uid="{1CBB1D75-2929-4283-8A12-6E05369FA01C}"/>
+    <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -170,6 +242,99 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>191505</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>105356</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{014A5201-C9DF-4A6E-83AA-ED520AB63F23}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9877425" y="704850"/>
+          <a:ext cx="7201905" cy="4163006"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>704849</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>284015</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2D993F3F-708A-447B-9BCA-D3B8273FA71C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="22402799" y="3371850"/>
+          <a:ext cx="3332016" cy="1266825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -435,94 +600,346 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B3:L6"/>
+  <dimension ref="B3:K6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-    </row>
-    <row r="4" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="E4" s="4">
+        <v>2025</v>
+      </c>
+      <c r="F4" s="4">
+        <v>2030</v>
+      </c>
+      <c r="G4" s="4">
+        <v>2035</v>
+      </c>
+      <c r="H4" s="4">
+        <v>2040</v>
+      </c>
+      <c r="I4" s="4">
+        <v>2045</v>
+      </c>
+      <c r="J4" s="4">
+        <v>2050</v>
+      </c>
+      <c r="K4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="4">
-        <v>2022</v>
-      </c>
-      <c r="F4" s="4">
-        <v>2025</v>
-      </c>
-      <c r="G4" s="4">
-        <v>2030</v>
-      </c>
-      <c r="H4" s="4">
-        <v>2035</v>
-      </c>
-      <c r="I4" s="4">
-        <v>2040</v>
-      </c>
-      <c r="J4" s="4">
-        <v>2045</v>
-      </c>
-      <c r="K4" s="4">
-        <v>2050</v>
-      </c>
-      <c r="L4" s="3" t="s">
+    </row>
+    <row r="5" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B5" s="5" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B5" s="5" t="s">
+      <c r="C5" s="5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="D6" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="E6">
+        <f>cite!AB5/1000</f>
+        <v>7.2999999999999995E-2</v>
+      </c>
+      <c r="F6">
+        <f>cite!AB6/1000</f>
+        <v>9.9873138444567022E-2</v>
+      </c>
+      <c r="G6">
+        <f>cite!AB7/1000</f>
+        <v>0.10512961941533369</v>
+      </c>
+      <c r="H6">
+        <f>cite!AB8/1000</f>
+        <v>0.10512961941533369</v>
+      </c>
+      <c r="I6">
+        <f>cite!AB9/1000</f>
+        <v>0.16820739106453392</v>
+      </c>
+      <c r="J6">
+        <f>cite!AB10/1000</f>
+        <v>0.19974627688913404</v>
+      </c>
+      <c r="K6" t="s">
         <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="D6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E6">
-        <v>0.08</v>
-      </c>
-      <c r="F6">
-        <v>7.2599999999999998E-2</v>
-      </c>
-      <c r="G6">
-        <v>0.08</v>
-      </c>
-      <c r="H6">
-        <v>8.6999999999999994E-2</v>
-      </c>
-      <c r="I6">
-        <v>8.6999999999999994E-2</v>
-      </c>
-      <c r="J6">
-        <v>8.6999999999999994E-2</v>
-      </c>
-      <c r="K6">
-        <v>8.6999999999999994E-2</v>
-      </c>
-      <c r="L6" t="s">
-        <v>8</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AF23FEF-5AD3-4D6A-BAA4-53FFF204BAEE}">
+  <dimension ref="O2:AD13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="2" spans="15:30" x14ac:dyDescent="0.25">
+      <c r="X2" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="15:30" x14ac:dyDescent="0.25">
+      <c r="Y3" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="Z3" s="7"/>
+      <c r="AA3" s="7"/>
+      <c r="AB3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="AC3" s="7"/>
+      <c r="AD3" s="7"/>
+    </row>
+    <row r="4" spans="15:30" x14ac:dyDescent="0.25">
+      <c r="P4" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>11</v>
+      </c>
+      <c r="R4" t="s">
+        <v>12</v>
+      </c>
+      <c r="S4" t="s">
+        <v>13</v>
+      </c>
+      <c r="T4" t="s">
+        <v>14</v>
+      </c>
+      <c r="X4" t="s">
+        <v>15</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>16</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>17</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>18</v>
+      </c>
+      <c r="AB4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AC4" t="s">
+        <v>17</v>
+      </c>
+      <c r="AD4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="15:30" x14ac:dyDescent="0.25">
+      <c r="O5">
+        <v>2035</v>
+      </c>
+      <c r="P5">
+        <v>174</v>
+      </c>
+      <c r="Q5">
+        <v>0.9244</v>
+      </c>
+      <c r="R5" s="8">
+        <f>P5*Q5</f>
+        <v>160.84559999999999</v>
+      </c>
+      <c r="S5" s="9">
+        <v>2.3E-2</v>
+      </c>
+      <c r="T5" s="10">
+        <f>R5*(1+S5)</f>
+        <v>164.54504879999999</v>
+      </c>
+      <c r="X5">
+        <v>2025</v>
+      </c>
+      <c r="AB5">
+        <v>73</v>
+      </c>
+      <c r="AC5">
+        <v>73</v>
+      </c>
+      <c r="AD5">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="6" spans="15:30" x14ac:dyDescent="0.25">
+      <c r="X6">
+        <v>2030</v>
+      </c>
+      <c r="Y6">
+        <v>95</v>
+      </c>
+      <c r="Z6">
+        <v>95</v>
+      </c>
+      <c r="AA6">
+        <v>73</v>
+      </c>
+      <c r="AB6" s="10">
+        <f>Y6*($V$13/$V$12)</f>
+        <v>99.873138444567019</v>
+      </c>
+      <c r="AC6" s="10">
+        <f>Z6*($V$13/$V$12)</f>
+        <v>99.873138444567019</v>
+      </c>
+      <c r="AD6" s="10">
+        <f>AA6*($V$13/$V$12)</f>
+        <v>76.744622173193605</v>
+      </c>
+    </row>
+    <row r="7" spans="15:30" x14ac:dyDescent="0.25">
+      <c r="X7">
+        <v>2035</v>
+      </c>
+      <c r="Y7">
+        <v>100</v>
+      </c>
+      <c r="Z7">
+        <v>140</v>
+      </c>
+      <c r="AA7">
+        <v>73</v>
+      </c>
+      <c r="AB7" s="10">
+        <f t="shared" ref="AB7:AB10" si="0">Y7*($V$13/$V$12)</f>
+        <v>105.12961941533369</v>
+      </c>
+      <c r="AC7" s="10">
+        <f t="shared" ref="AC7:AC10" si="1">Z7*($V$13/$V$12)</f>
+        <v>147.18146718146718</v>
+      </c>
+      <c r="AD7" s="10">
+        <f t="shared" ref="AD7:AD10" si="2">AA7*($V$13/$V$12)</f>
+        <v>76.744622173193605</v>
+      </c>
+    </row>
+    <row r="8" spans="15:30" x14ac:dyDescent="0.25">
+      <c r="X8">
+        <v>2040</v>
+      </c>
+      <c r="Y8">
+        <v>100</v>
+      </c>
+      <c r="Z8">
+        <v>290</v>
+      </c>
+      <c r="AA8">
+        <v>73</v>
+      </c>
+      <c r="AB8" s="10">
+        <f t="shared" si="0"/>
+        <v>105.12961941533369</v>
+      </c>
+      <c r="AC8" s="10">
+        <f t="shared" si="1"/>
+        <v>304.87589630446774</v>
+      </c>
+      <c r="AD8" s="10">
+        <f t="shared" si="2"/>
+        <v>76.744622173193605</v>
+      </c>
+    </row>
+    <row r="9" spans="15:30" x14ac:dyDescent="0.25">
+      <c r="X9">
+        <v>2045</v>
+      </c>
+      <c r="Y9">
+        <v>160</v>
+      </c>
+      <c r="Z9">
+        <v>430</v>
+      </c>
+      <c r="AA9">
+        <v>73</v>
+      </c>
+      <c r="AB9" s="10">
+        <f t="shared" si="0"/>
+        <v>168.20739106453391</v>
+      </c>
+      <c r="AC9" s="10">
+        <f t="shared" si="1"/>
+        <v>452.0573634859349</v>
+      </c>
+      <c r="AD9" s="10">
+        <f t="shared" si="2"/>
+        <v>76.744622173193605</v>
+      </c>
+    </row>
+    <row r="10" spans="15:30" x14ac:dyDescent="0.25">
+      <c r="X10">
+        <v>2050</v>
+      </c>
+      <c r="Y10">
+        <v>190</v>
+      </c>
+      <c r="Z10">
+        <v>490</v>
+      </c>
+      <c r="AA10">
+        <v>73</v>
+      </c>
+      <c r="AB10" s="10">
+        <f t="shared" si="0"/>
+        <v>199.74627688913404</v>
+      </c>
+      <c r="AC10" s="10">
+        <f t="shared" si="1"/>
+        <v>515.1351351351351</v>
+      </c>
+      <c r="AD10" s="10">
+        <f t="shared" si="2"/>
+        <v>76.744622173193605</v>
+      </c>
+    </row>
+    <row r="12" spans="15:30" x14ac:dyDescent="0.25">
+      <c r="U12" t="s">
+        <v>19</v>
+      </c>
+      <c r="V12">
+        <v>126.91</v>
+      </c>
+    </row>
+    <row r="13" spans="15:30" x14ac:dyDescent="0.25">
+      <c r="U13" t="s">
+        <v>20</v>
+      </c>
+      <c r="V13">
+        <v>133.41999999999999</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="Y3:AA3"/>
+    <mergeCell ref="AB3:AD3"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="X2" r:id="rId1" display="https://www.eionet.europa.eu/etcs/etc-cm/products/etc-cm-report-2025-06/@@download/file/ETS-Report_2025_final.pdf" xr:uid="{FCAB02CA-783C-42B9-9133-A467F919A18D}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Adding flo_cost to fuels
</commit_message>
<xml_diff>
--- a/SuppXLS/Scen_CO2_price.xlsx
+++ b/SuppXLS/Scen_CO2_price.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86F3D1C2-2CC4-4EAB-98CA-795028B2C2B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D26D0DF-BC7C-4621-A67F-7B9617CD3280}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,6 +39,9 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="23">
   <si>
+    <t>~TFM_INS-TS</t>
+  </si>
+  <si>
     <t>TimeSlice</t>
   </si>
   <si>
@@ -103,9 +106,6 @@
   </si>
   <si>
     <t>eur25/kt</t>
-  </si>
-  <si>
-    <t>~TFM_INS</t>
   </si>
 </sst>
 </file>
@@ -609,20 +609,20 @@
   <sheetData>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
     </row>
     <row r="4" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="3" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E4" s="4">
         <v>2025</v>
@@ -643,20 +643,20 @@
         <v>2050</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B5" s="5" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6" spans="2:11" x14ac:dyDescent="0.25">
       <c r="D6" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E6">
         <f>cite!AB5/1000</f>
@@ -683,7 +683,7 @@
         <v>0.19974627688913404</v>
       </c>
       <c r="K6" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -698,57 +698,57 @@
   <sheetData>
     <row r="2" spans="15:30" x14ac:dyDescent="0.25">
       <c r="X2" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="15:30" x14ac:dyDescent="0.25">
       <c r="Y3" s="7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Z3" s="7"/>
       <c r="AA3" s="7"/>
       <c r="AB3" s="7" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AC3" s="7"/>
       <c r="AD3" s="7"/>
     </row>
     <row r="4" spans="15:30" x14ac:dyDescent="0.25">
       <c r="P4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Q4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="R4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="S4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="T4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="Y4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="Z4" t="s">
+        <v>18</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>19</v>
+      </c>
+      <c r="AB4" t="s">
         <v>17</v>
       </c>
-      <c r="AA4" t="s">
+      <c r="AC4" t="s">
         <v>18</v>
       </c>
-      <c r="AB4" t="s">
-        <v>16</v>
-      </c>
-      <c r="AC4" t="s">
-        <v>17</v>
-      </c>
       <c r="AD4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="15:30" x14ac:dyDescent="0.25">
@@ -917,7 +917,7 @@
     </row>
     <row r="12" spans="15:30" x14ac:dyDescent="0.25">
       <c r="U12" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="V12">
         <v>126.91</v>
@@ -925,7 +925,7 @@
     </row>
     <row r="13" spans="15:30" x14ac:dyDescent="0.25">
       <c r="U13" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="V13">
         <v>133.41999999999999</v>

</xml_diff>

<commit_message>
Kill gas plants scen
</commit_message>
<xml_diff>
--- a/SuppXLS/Scen_CO2_price.xlsx
+++ b/SuppXLS/Scen_CO2_price.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D26D0DF-BC7C-4621-A67F-7B9617CD3280}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F30397E7-AB6A-4E29-81DA-237126973235}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CO2" sheetId="1" r:id="rId1"/>
@@ -105,7 +105,7 @@
     <t>HICP_2025</t>
   </si>
   <si>
-    <t>eur25/kt</t>
+    <t>Meur25/kt</t>
   </si>
 </sst>
 </file>
@@ -218,12 +218,12 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="3"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hyperlink" xfId="3" builtinId="8"/>
@@ -604,6 +604,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -702,16 +703,16 @@
       </c>
     </row>
     <row r="3" spans="15:30" x14ac:dyDescent="0.25">
-      <c r="Y3" s="7" t="s">
+      <c r="Y3" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="Z3" s="7"/>
-      <c r="AA3" s="7"/>
-      <c r="AB3" s="7" t="s">
+      <c r="Z3" s="10"/>
+      <c r="AA3" s="10"/>
+      <c r="AB3" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="AC3" s="7"/>
-      <c r="AD3" s="7"/>
+      <c r="AC3" s="10"/>
+      <c r="AD3" s="10"/>
     </row>
     <row r="4" spans="15:30" x14ac:dyDescent="0.25">
       <c r="P4" t="s">
@@ -761,14 +762,14 @@
       <c r="Q5">
         <v>0.9244</v>
       </c>
-      <c r="R5" s="8">
+      <c r="R5" s="7">
         <f>P5*Q5</f>
         <v>160.84559999999999</v>
       </c>
-      <c r="S5" s="9">
+      <c r="S5" s="8">
         <v>2.3E-2</v>
       </c>
-      <c r="T5" s="10">
+      <c r="T5" s="9">
         <f>R5*(1+S5)</f>
         <v>164.54504879999999</v>
       </c>
@@ -798,15 +799,15 @@
       <c r="AA6">
         <v>73</v>
       </c>
-      <c r="AB6" s="10">
+      <c r="AB6" s="9">
         <f>Y6*($V$13/$V$12)</f>
         <v>99.873138444567019</v>
       </c>
-      <c r="AC6" s="10">
+      <c r="AC6" s="9">
         <f>Z6*($V$13/$V$12)</f>
         <v>99.873138444567019</v>
       </c>
-      <c r="AD6" s="10">
+      <c r="AD6" s="9">
         <f>AA6*($V$13/$V$12)</f>
         <v>76.744622173193605</v>
       </c>
@@ -824,15 +825,15 @@
       <c r="AA7">
         <v>73</v>
       </c>
-      <c r="AB7" s="10">
+      <c r="AB7" s="9">
         <f t="shared" ref="AB7:AB10" si="0">Y7*($V$13/$V$12)</f>
         <v>105.12961941533369</v>
       </c>
-      <c r="AC7" s="10">
+      <c r="AC7" s="9">
         <f t="shared" ref="AC7:AC10" si="1">Z7*($V$13/$V$12)</f>
         <v>147.18146718146718</v>
       </c>
-      <c r="AD7" s="10">
+      <c r="AD7" s="9">
         <f t="shared" ref="AD7:AD10" si="2">AA7*($V$13/$V$12)</f>
         <v>76.744622173193605</v>
       </c>
@@ -850,15 +851,15 @@
       <c r="AA8">
         <v>73</v>
       </c>
-      <c r="AB8" s="10">
+      <c r="AB8" s="9">
         <f t="shared" si="0"/>
         <v>105.12961941533369</v>
       </c>
-      <c r="AC8" s="10">
+      <c r="AC8" s="9">
         <f t="shared" si="1"/>
         <v>304.87589630446774</v>
       </c>
-      <c r="AD8" s="10">
+      <c r="AD8" s="9">
         <f t="shared" si="2"/>
         <v>76.744622173193605</v>
       </c>
@@ -876,15 +877,15 @@
       <c r="AA9">
         <v>73</v>
       </c>
-      <c r="AB9" s="10">
+      <c r="AB9" s="9">
         <f t="shared" si="0"/>
         <v>168.20739106453391</v>
       </c>
-      <c r="AC9" s="10">
+      <c r="AC9" s="9">
         <f t="shared" si="1"/>
         <v>452.0573634859349</v>
       </c>
-      <c r="AD9" s="10">
+      <c r="AD9" s="9">
         <f t="shared" si="2"/>
         <v>76.744622173193605</v>
       </c>
@@ -902,15 +903,15 @@
       <c r="AA10">
         <v>73</v>
       </c>
-      <c r="AB10" s="10">
+      <c r="AB10" s="9">
         <f t="shared" si="0"/>
         <v>199.74627688913404</v>
       </c>
-      <c r="AC10" s="10">
+      <c r="AC10" s="9">
         <f t="shared" si="1"/>
         <v>515.1351351351351</v>
       </c>
-      <c r="AD10" s="10">
+      <c r="AD10" s="9">
         <f t="shared" si="2"/>
         <v>76.744622173193605</v>
       </c>

</xml_diff>